<commit_message>
Capture all CBP bulletin columns, not just liquidation date
Output now mirrors the CBP bulletin table: one row per matter with
Event Type; per-event-type date columns (Liquidation, Re-liquidation,
Extension, Suspension) so multi-event entries keep every date; plus
Posted/Voided Date, Basis, Action, Port, Entry Date/Type, Team, Filer.
Parsing keys off CBP event codes (L/R/E/S). Added summary metrics for
entries carrying a re-liquidation, extension, or suspension.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Liquidation_Date_Auto/SAMPLE_output.xlsx
+++ b/Liquidation_Date_Auto/SAMPLE_output.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,12 +429,77 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Lookup Status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Event Type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Liquidation Date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Lookup Status</t>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Re-liquidation Date</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Extension Date</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Suspension Date</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Posted Date</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Voided Date</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Port of Entry</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Entry Date</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Entry Type</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Filer</t>
         </is>
       </c>
     </row>
@@ -451,12 +516,57 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>LIQUIDATED</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Liquidated</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>LIQUIDATED</t>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>No Change</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>5401</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2025-08-18</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>GBM</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>E86</t>
         </is>
       </c>
     </row>
@@ -473,12 +583,57 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>LIQUIDATED</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Liquidated</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>LIQUIDATED</t>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>No Change</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>4197</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2025-08-18</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>GBQ</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>E86</t>
         </is>
       </c>
     </row>
@@ -495,12 +650,57 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>LIQUIDATED</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Liquidated</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>LIQUIDATED</t>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>No Change</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0401</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2025-08-18</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>EBF</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>E86</t>
         </is>
       </c>
     </row>
@@ -517,12 +717,57 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>LIQUIDATED</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Liquidated</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>LIQUIDATED</t>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>No Change</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>0417</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2025-08-11</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>GBQ</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>E86</t>
         </is>
       </c>
     </row>
@@ -539,12 +784,57 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>LIQUIDATED</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Liquidated</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>LIQUIDATED</t>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>No Change</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>5401</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2025-08-18</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>GBM</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>E86</t>
         </is>
       </c>
     </row>
@@ -559,12 +849,25 @@
           <t>99999999999</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>NOT FOUND (no bulletin notice for this entry)</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -579,12 +882,57 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>LIQUIDATED</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Liquidated</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>LIQUIDATED</t>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>No Change</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>0417</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2025-08-11</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>JBK</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>E86</t>
         </is>
       </c>
     </row>
@@ -595,12 +943,25 @@
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>EMPTY (no entry number in this row)</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -615,12 +976,57 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>LIQUIDATED</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Liquidated</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>LIQUIDATED</t>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>No Change</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>4772</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2025-08-07</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>GBM</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>E86</t>
         </is>
       </c>
     </row>
@@ -637,12 +1043,57 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>LIQUIDATED</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Liquidated</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>LIQUIDATED</t>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>No Change</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>0401</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2025-08-07</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>EBF</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>E86</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Output dates in US format (MM/DD/YYYY)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Liquidation_Date_Auto/SAMPLE_output.xlsx
+++ b/Liquidation_Date_Auto/SAMPLE_output.xlsx
@@ -526,7 +526,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -534,7 +534,7 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -551,7 +551,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2025-08-18</t>
+          <t>08/18/2025</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -601,7 +601,7 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -618,7 +618,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2025-08-18</t>
+          <t>08/18/2025</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -668,7 +668,7 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -685,7 +685,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2025-08-18</t>
+          <t>08/18/2025</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -735,7 +735,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -752,7 +752,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2025-08-11</t>
+          <t>08/11/2025</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -802,7 +802,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -819,7 +819,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2025-08-18</t>
+          <t>08/18/2025</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -900,7 +900,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -917,7 +917,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2025-08-11</t>
+          <t>08/11/2025</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -994,7 +994,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>2025-08-07</t>
+          <t>08/07/2025</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -1061,7 +1061,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>07/03/2026</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>2025-08-07</t>
+          <t>08/07/2025</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">

</xml_diff>

<commit_message>
Revert "Output dates in US format (MM/DD/YYYY)"
This reverts commit df2c2429b921e8722639a35e3e701d94baae50b9.
</commit_message>
<xml_diff>
--- a/Liquidation_Date_Auto/SAMPLE_output.xlsx
+++ b/Liquidation_Date_Auto/SAMPLE_output.xlsx
@@ -526,7 +526,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -534,7 +534,7 @@
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -551,7 +551,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>08/18/2025</t>
+          <t>2025-08-18</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -601,7 +601,7 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -618,7 +618,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>08/18/2025</t>
+          <t>2025-08-18</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -668,7 +668,7 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -685,7 +685,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>08/18/2025</t>
+          <t>2025-08-18</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -735,7 +735,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -752,7 +752,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>08/11/2025</t>
+          <t>2025-08-11</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -802,7 +802,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -819,7 +819,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>08/18/2025</t>
+          <t>2025-08-18</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -900,7 +900,7 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -917,7 +917,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>08/11/2025</t>
+          <t>2025-08-11</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -994,7 +994,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>08/07/2025</t>
+          <t>2025-08-07</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -1061,7 +1061,7 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>07/03/2026</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>08/07/2025</t>
+          <t>2025-08-07</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">

</xml_diff>

<commit_message>
Write output dates as real Excel dates formatted yyyy-mm-dd
Plain-text dates could be re-rendered by Excel in the viewer's regional
format (e.g. DD/MM/YYYY); a fixed number format keeps them as yyyy-mm-dd.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Liquidation_Date_Auto/SAMPLE_output.xlsx
+++ b/Liquidation_Date_Auto/SAMPLE_output.xlsx
@@ -16,7 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -524,20 +529,16 @@
           <t>Liquidated</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="E2" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F2" s="1" t="inlineStr"/>
+      <c r="G2" s="1" t="inlineStr"/>
+      <c r="H2" s="1" t="inlineStr"/>
+      <c r="I2" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="J2" s="1" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
@@ -549,10 +550,8 @@
           <t>5401</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>2025-08-18</t>
-        </is>
+      <c r="N2" s="1" t="n">
+        <v>45887</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -591,20 +590,16 @@
           <t>Liquidated</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="E3" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F3" s="1" t="inlineStr"/>
+      <c r="G3" s="1" t="inlineStr"/>
+      <c r="H3" s="1" t="inlineStr"/>
+      <c r="I3" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="J3" s="1" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
@@ -616,10 +611,8 @@
           <t>4197</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2025-08-18</t>
-        </is>
+      <c r="N3" s="1" t="n">
+        <v>45887</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -658,20 +651,16 @@
           <t>Liquidated</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="E4" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F4" s="1" t="inlineStr"/>
+      <c r="G4" s="1" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr"/>
+      <c r="I4" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="J4" s="1" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
@@ -683,10 +672,8 @@
           <t>0401</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2025-08-18</t>
-        </is>
+      <c r="N4" s="1" t="n">
+        <v>45887</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -725,20 +712,16 @@
           <t>Liquidated</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="E5" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="F5" s="1" t="inlineStr"/>
+      <c r="G5" s="1" t="inlineStr"/>
+      <c r="H5" s="1" t="inlineStr"/>
+      <c r="I5" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="J5" s="1" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
@@ -750,10 +733,8 @@
           <t>0417</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2025-08-11</t>
-        </is>
+      <c r="N5" s="1" t="n">
+        <v>45880</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -792,20 +773,16 @@
           <t>Liquidated</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-07-10</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="E6" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="F6" s="1" t="inlineStr"/>
+      <c r="G6" s="1" t="inlineStr"/>
+      <c r="H6" s="1" t="inlineStr"/>
+      <c r="I6" s="1" t="n">
+        <v>46213</v>
+      </c>
+      <c r="J6" s="1" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
@@ -817,10 +794,8 @@
           <t>5401</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>2025-08-18</t>
-        </is>
+      <c r="N6" s="1" t="n">
+        <v>45887</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -855,16 +830,16 @@
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
+      <c r="E7" s="1" t="inlineStr"/>
+      <c r="F7" s="1" t="inlineStr"/>
+      <c r="G7" s="1" t="inlineStr"/>
+      <c r="H7" s="1" t="inlineStr"/>
+      <c r="I7" s="1" t="inlineStr"/>
+      <c r="J7" s="1" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
+      <c r="N7" s="1" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
@@ -890,20 +865,16 @@
           <t>Liquidated</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
+      <c r="E8" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="F8" s="1" t="inlineStr"/>
+      <c r="G8" s="1" t="inlineStr"/>
+      <c r="H8" s="1" t="inlineStr"/>
+      <c r="I8" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="J8" s="1" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
@@ -915,10 +886,8 @@
           <t>0417</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>2025-08-11</t>
-        </is>
+      <c r="N8" s="1" t="n">
+        <v>45880</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -949,16 +918,16 @@
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
+      <c r="E9" s="1" t="inlineStr"/>
+      <c r="F9" s="1" t="inlineStr"/>
+      <c r="G9" s="1" t="inlineStr"/>
+      <c r="H9" s="1" t="inlineStr"/>
+      <c r="I9" s="1" t="inlineStr"/>
+      <c r="J9" s="1" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" s="1" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
@@ -984,20 +953,16 @@
           <t>Liquidated</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="E10" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="F10" s="1" t="inlineStr"/>
+      <c r="G10" s="1" t="inlineStr"/>
+      <c r="H10" s="1" t="inlineStr"/>
+      <c r="I10" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="J10" s="1" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
@@ -1009,10 +974,8 @@
           <t>4772</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>2025-08-07</t>
-        </is>
+      <c r="N10" s="1" t="n">
+        <v>45876</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1051,20 +1014,16 @@
           <t>Liquidated</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="E11" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="F11" s="1" t="inlineStr"/>
+      <c r="G11" s="1" t="inlineStr"/>
+      <c r="H11" s="1" t="inlineStr"/>
+      <c r="I11" s="1" t="n">
+        <v>46206</v>
+      </c>
+      <c r="J11" s="1" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
@@ -1076,10 +1035,8 @@
           <t>0401</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>2025-08-07</t>
-        </is>
+      <c r="N11" s="1" t="n">
+        <v>45876</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>

</xml_diff>